<commit_message>
chore(bancos): atualiza bases de dados utilizados no projetos para ploa2025-substitutivo
See #163
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_QDD_FISCAL_FONTE_95.xlsx
+++ b/bancos/SISOR/BASE_QDD_FISCAL_FONTE_95.xlsx
@@ -616,7 +616,7 @@
         <v>39</v>
       </c>
       <c r="L2" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M2" t="n">
         <v>1</v>
@@ -732,7 +732,7 @@
         <v>39</v>
       </c>
       <c r="L3" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M3" t="n">
         <v>1</v>
@@ -848,7 +848,7 @@
         <v>39</v>
       </c>
       <c r="L4" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M4" t="n">
         <v>1</v>
@@ -964,7 +964,7 @@
         <v>39</v>
       </c>
       <c r="L5" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M5" t="n">
         <v>1</v>
@@ -1080,7 +1080,7 @@
         <v>39</v>
       </c>
       <c r="L6" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M6" t="n">
         <v>1</v>
@@ -1196,7 +1196,7 @@
         <v>39</v>
       </c>
       <c r="L7" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M7" t="n">
         <v>1</v>
@@ -1312,7 +1312,7 @@
         <v>39</v>
       </c>
       <c r="L8" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M8" t="n">
         <v>1</v>
@@ -1428,7 +1428,7 @@
         <v>52</v>
       </c>
       <c r="L9" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M9" t="n">
         <v>1</v>
@@ -1544,7 +1544,7 @@
         <v>39</v>
       </c>
       <c r="L10" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M10" t="n">
         <v>1</v>
@@ -1660,7 +1660,7 @@
         <v>39</v>
       </c>
       <c r="L11" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M11" t="n">
         <v>1</v>
@@ -1890,7 +1890,7 @@
         <v>39</v>
       </c>
       <c r="L13" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M13" t="n">
         <v>1</v>
@@ -2462,7 +2462,7 @@
         <v>39</v>
       </c>
       <c r="L18" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M18" t="n">
         <v>1</v>
@@ -2578,7 +2578,7 @@
         <v>39</v>
       </c>
       <c r="L19" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M19" t="n">
         <v>1</v>
@@ -2694,7 +2694,7 @@
         <v>39</v>
       </c>
       <c r="L20" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M20" t="n">
         <v>1</v>
@@ -2810,7 +2810,7 @@
         <v>39</v>
       </c>
       <c r="L21" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M21" t="n">
         <v>1</v>
@@ -2926,7 +2926,7 @@
         <v>39</v>
       </c>
       <c r="L22" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M22" t="n">
         <v>1</v>
@@ -3042,7 +3042,7 @@
         <v>39</v>
       </c>
       <c r="L23" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M23" t="n">
         <v>1</v>
@@ -3158,7 +3158,7 @@
         <v>39</v>
       </c>
       <c r="L24" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M24" t="n">
         <v>1</v>
@@ -3274,7 +3274,7 @@
         <v>39</v>
       </c>
       <c r="L25" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M25" t="n">
         <v>1</v>
@@ -3390,7 +3390,7 @@
         <v>39</v>
       </c>
       <c r="L26" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M26" t="n">
         <v>1</v>
@@ -3506,7 +3506,7 @@
         <v>52</v>
       </c>
       <c r="L27" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M27" t="n">
         <v>1</v>
@@ -3622,7 +3622,7 @@
         <v>52</v>
       </c>
       <c r="L28" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M28" t="n">
         <v>1</v>
@@ -3738,7 +3738,7 @@
         <v>39</v>
       </c>
       <c r="L29" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M29" t="n">
         <v>1</v>
@@ -3854,7 +3854,7 @@
         <v>39</v>
       </c>
       <c r="L30" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M30" t="n">
         <v>1</v>
@@ -3970,7 +3970,7 @@
         <v>39</v>
       </c>
       <c r="L31" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M31" t="n">
         <v>1</v>
@@ -4086,7 +4086,7 @@
         <v>39</v>
       </c>
       <c r="L32" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M32" t="n">
         <v>1</v>
@@ -4202,7 +4202,7 @@
         <v>39</v>
       </c>
       <c r="L33" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M33" t="n">
         <v>1</v>
@@ -4318,7 +4318,7 @@
         <v>39</v>
       </c>
       <c r="L34" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M34" t="n">
         <v>1</v>
@@ -4548,7 +4548,7 @@
         <v>39</v>
       </c>
       <c r="L36" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M36" t="n">
         <v>1</v>
@@ -4664,7 +4664,7 @@
         <v>39</v>
       </c>
       <c r="L37" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M37" t="n">
         <v>1</v>
@@ -4780,7 +4780,7 @@
         <v>52</v>
       </c>
       <c r="L38" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M38" t="n">
         <v>1</v>
@@ -4896,7 +4896,7 @@
         <v>65</v>
       </c>
       <c r="L39" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M39" t="n">
         <v>1</v>

</xml_diff>